<commit_message>
Handover: record the battery case and what feeds it
A third case exists as of today, and the handover said there were two. It does
not change NEXT -- the model is still finished and the numbers are still what is
missing -- but it adds 66 empty rows to that count, and it names where its
inflow comes from and in what unit.

It also records the one thing about this case that is not like the others: two
of the chemistries it carries have no described cell. Sodium-ion's holds no CRM
or SRM, so its absence costs a recovery answer nothing. Solid-state's holds
lithium, and no coefficient can be written for a composition that does not
exist.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/params.xlsx
+++ b/params.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D34"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -502,7 +502,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2020-2070, 1</t>
+          <t>2020-2070, 5</t>
         </is>
       </c>
     </row>
@@ -1031,116 +1031,6 @@
       <c r="D29" t="inlineStr">
         <is>
           <t>["copper"]</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>cases</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>WHICH CASES ARE ADDED. Any number; battery packs and drivetrains join by being listed here once they have a case folder of their own. SAFE TO CHANGE: yes. A folder that does not exist is named and refused.</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>combine.cases</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>["data_folder/bev_electronics_wiring", "data_folder/bev_electronics_boards"]</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>resource</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>THE METAL, AS EACH CASE NAMES IT. The wiring case resolves materials and calls it `copper`; the boards case resolves elements and calls it `Cu`. They are the same metal, and this is the only place that says so -- every name listed is looked for in every case, and whichever one that case has is the one used. SAFE TO CHANGE: yes. A case with none of these names is reported as contributing nothing rather than silently counting zero.</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>combine.resource</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>["copper", "Cu"]</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>label</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>What the metal is called in the title. The names above are how the data spells it; this is how a reader says it. SAFE TO CHANGE: yes.</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>combine.label</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>copper</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>whole</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>What the combined streams are called together, for the title. SAFE TO CHANGE: yes.</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>combine.whole</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>BEV electronics</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>out_dir</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>WHERE THE COMBINED FIGURE GOES. Not any one case's folder: it belongs to none of them. SAFE TO CHANGE: yes.</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>combine.out_dir</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>figures/combined</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
05 combines the five battery cases, and a case leaves a pass it has no scenario for
The first run of 05 after the study stopped at S2: data/battery is refused by its
own input check once the export carries the sodium cells (Na, P, C and
batteryCellUnitemised have no coefficient in it). On his word "Yes, do 1 and 2":

combine.cases lists LFP, LMFP, NMC_high, sodium and solid-state in place of
data/battery, and upstream.offers_scenario leaves a case out of a pass it has no
scenario for (sodium in S1, solid-state in S1 and S2) with a printed line, as a
case that cannot carry the metal already was. The first case listed with scenarios
still decides the passes, so LFP comes first. Two tests, red then green; a
single-case check at 200 draws; 165 tests pass. DECISIONS 53, BATTERY_ROUTES 13.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/params.xlsx
+++ b/params.xlsx
@@ -1064,7 +1064,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>WHICH CASES ARE ADDED. Any number; battery packs and drivetrains join by being listed here once they have a case folder of their own. SAFE TO CHANGE: yes. A folder that does not exist is named and refused.</t>
+          <t>WHICH CASES ARE ADDED. Any number; battery packs and drivetrains join by being listed here once they have a case folder of their own. SAFE TO CHANGE: yes. A folder that does not exist is named and refused.  THE BATTERY IS FIVE CASES, one per chemistry (2026-10-09; `data/battery`, the one blended case, is no longer here: its input check refuses S2 and S3, which carry the sodium cells). A case that does not have the scenario of a pass -- sodium has no S1, solid-state has neither S1 nor S2 -- is left out of that pass with a line saying so, so the three scenarios add three, four and five battery cases in turn. THE FIRST CASE LISTED THAT HAS SCENARIOS DECIDES WHICH PASSES ARE MADE, so the one that has all of them (LFP) comes first of the battery cases. Put sodium first and S1 is not run.</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1074,7 +1074,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>["data/bev_electronics_wiring", "data/bev_electronics_boards", "data/battery", "data/tractionmotor"]</t>
+          <t>["data/bev_electronics_wiring", "data/bev_electronics_boards", "data/battery_lfp", "data/battery_lmfp", "data/battery_nmc_high", "data/battery_sodium", "data/battery_solid_state", "data/tractionmotor"]</t>
         </is>
       </c>
     </row>

</xml_diff>